<commit_message>
checkpoint before report engine redesign CP 14.4
</commit_message>
<xml_diff>
--- a/SynOS_Catalog_Master_Template.xlsx
+++ b/SynOS_Catalog_Master_Template.xlsx
@@ -966,7 +966,6 @@
           <t>True</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Fasting Glucose</t>
@@ -997,7 +996,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1040,7 +1038,6 @@
           <t>True</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Total Bilirubin</t>
@@ -1071,7 +1068,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1210,7 +1206,6 @@
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>True</t>
@@ -1253,19 +1248,16 @@
           <t>1.2</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>True</t>

</xml_diff>